<commit_message>
update the excel template
</commit_message>
<xml_diff>
--- a/V-COORDINATE--Scheduled.xlsx
+++ b/V-COORDINATE--Scheduled.xlsx
@@ -5,108 +5,32 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://chenoafundorg-my.sharepoint.com/personal/anthony_child_chenoafund_org/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anthony.Child\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="229" documentId="13_ncr:1_{9715ABA8-DA3B-48A0-8204-36B144813BB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1931922C-2139-4329-B201-F5386FF45FD1}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2316F981-2EC3-4E22-A5E3-6D7CCB3D09A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C0061742-0291-45E3-9652-9BB2CC5C9823}"/>
+    <workbookView xWindow="3360" yWindow="1395" windowWidth="20910" windowHeight="19275" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="AM1" sheetId="13" r:id="rId1"/>
-    <sheet name="PM1" sheetId="14" r:id="rId2"/>
-    <sheet name="Sheet1" sheetId="12" r:id="rId3"/>
+    <sheet name="AM1" sheetId="1" r:id="rId1"/>
+    <sheet name="PM1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'AM1'!$B$1:$BK$31</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'PM1'!$B$1:$BK$31</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="38">
   <si>
-    <t>Off.</t>
-  </si>
-  <si>
-    <t>Live?</t>
-  </si>
-  <si>
-    <t>Language?</t>
-  </si>
-  <si>
-    <t>Other?</t>
-  </si>
-  <si>
-    <t>Wchr/Wlkr?</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>5P</t>
-  </si>
-  <si>
-    <t>6P</t>
-  </si>
-  <si>
-    <t>7P</t>
-  </si>
-  <si>
-    <t>8P</t>
-  </si>
-  <si>
-    <t>Narrow Side?</t>
-  </si>
-  <si>
-    <t>S</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>(#2/#3)</t>
-  </si>
-  <si>
-    <t>(#6/#7)</t>
-  </si>
-  <si>
     <t>A.M.</t>
   </si>
   <si>
-    <t>P.M.</t>
-  </si>
-  <si>
-    <t>S:</t>
-  </si>
-  <si>
-    <t>Skip V6 if possible</t>
-  </si>
-  <si>
-    <t>Skip V3 if possible</t>
-  </si>
-  <si>
-    <t>THIN RECEIVERS</t>
-  </si>
-  <si>
-    <t>Low voice, Gentle,
-Reverence, 5 Min</t>
-  </si>
-  <si>
-    <t>B:</t>
-  </si>
-  <si>
-    <t>Off:</t>
-  </si>
-  <si>
-    <t>Bros Available?</t>
+    <t>Room:</t>
   </si>
   <si>
     <t>Time:</t>
@@ -127,6 +51,82 @@
     <t xml:space="preserve"> 1:00+</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
+    <t>B:</t>
+  </si>
+  <si>
+    <t>S:</t>
+  </si>
+  <si>
+    <t>Off:</t>
+  </si>
+  <si>
+    <t>AM Shift</t>
+  </si>
+  <si>
+    <t>5P</t>
+  </si>
+  <si>
+    <t>6P</t>
+  </si>
+  <si>
+    <t>7P</t>
+  </si>
+  <si>
+    <t>8P</t>
+  </si>
+  <si>
+    <t>Off.</t>
+  </si>
+  <si>
+    <t>Low voice, Gentle,
+Reverence, 5 Min</t>
+  </si>
+  <si>
+    <t>Skip V6 if possible</t>
+  </si>
+  <si>
+    <t>Skip V3 if possible</t>
+  </si>
+  <si>
+    <t>Bros Available?</t>
+  </si>
+  <si>
+    <t>Narrow Side?</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>THIN RECEIVERS</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>Live?</t>
+  </si>
+  <si>
+    <t>Wchr/Wlkr?</t>
+  </si>
+  <si>
+    <t>(#2/#3)</t>
+  </si>
+  <si>
+    <t>(#6/#7)</t>
+  </si>
+  <si>
+    <t>Language?</t>
+  </si>
+  <si>
+    <t>Other?</t>
+  </si>
+  <si>
+    <t>P.M.</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 2:00+</t>
   </si>
   <si>
@@ -140,12 +140,6 @@
   </si>
   <si>
     <t xml:space="preserve"> 4:00+</t>
-  </si>
-  <si>
-    <t>Room:</t>
-  </si>
-  <si>
-    <t>AM Shift</t>
   </si>
 </sst>
 </file>
@@ -239,13 +233,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="4" tint="-0.249977111117893"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -263,6 +250,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF335593"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="7">
@@ -303,7 +296,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="50">
+  <borders count="54">
     <border>
       <left/>
       <right/>
@@ -625,19 +618,6 @@
       <right style="medium">
         <color auto="1"/>
       </right>
-      <top style="double">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -668,17 +648,6 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -762,19 +731,6 @@
         <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="double">
         <color auto="1"/>
       </bottom>
       <diagonal/>
@@ -914,11 +870,108 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="double">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="double">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="double">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="double">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="double">
+        <color auto="1"/>
+      </top>
+      <bottom style="double">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="double">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
@@ -962,7 +1015,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
@@ -978,19 +1031,19 @@
     <xf numFmtId="49" fontId="0" fillId="5" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="33" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="31" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="34" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="32" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="35" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="33" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1003,175 +1056,126 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="49" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="49" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <mruColors>
-      <color rgb="FFCCFFFF"/>
-      <color rgb="FFFF3300"/>
-      <color rgb="FFFF6600"/>
-    </mruColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1479,7 +1483,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE1F9E79-6852-4F92-A3A8-EA17B75FA31C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BL32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1489,11 +1493,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:64" ht="17.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="C1" s="78" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="62" t="s">
-        <v>36</v>
+      <c r="C1" s="83" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="72" t="s">
+        <v>1</v>
       </c>
       <c r="E1" s="63"/>
       <c r="F1" s="63"/>
@@ -1501,15 +1505,15 @@
       <c r="H1" s="63"/>
       <c r="I1" s="63"/>
       <c r="J1" s="63"/>
-      <c r="K1" s="64">
+      <c r="K1" s="86">
         <v>1</v>
       </c>
-      <c r="L1" s="64"/>
-      <c r="M1" s="64"/>
-      <c r="N1" s="64"/>
-      <c r="O1" s="65"/>
-      <c r="P1" s="63" t="s">
-        <v>36</v>
+      <c r="L1" s="63"/>
+      <c r="M1" s="63"/>
+      <c r="N1" s="63"/>
+      <c r="O1" s="87"/>
+      <c r="P1" s="62" t="s">
+        <v>1</v>
       </c>
       <c r="Q1" s="63"/>
       <c r="R1" s="63"/>
@@ -1517,15 +1521,15 @@
       <c r="T1" s="63"/>
       <c r="U1" s="63"/>
       <c r="V1" s="63"/>
-      <c r="W1" s="64">
+      <c r="W1" s="78">
         <v>2</v>
       </c>
-      <c r="X1" s="64"/>
-      <c r="Y1" s="64"/>
-      <c r="Z1" s="64"/>
-      <c r="AA1" s="64"/>
-      <c r="AB1" s="66" t="s">
-        <v>36</v>
+      <c r="X1" s="63"/>
+      <c r="Y1" s="63"/>
+      <c r="Z1" s="63"/>
+      <c r="AA1" s="63"/>
+      <c r="AB1" s="64" t="s">
+        <v>1</v>
       </c>
       <c r="AC1" s="63"/>
       <c r="AD1" s="63"/>
@@ -1533,15 +1537,15 @@
       <c r="AF1" s="63"/>
       <c r="AG1" s="63"/>
       <c r="AH1" s="63"/>
-      <c r="AI1" s="64">
+      <c r="AI1" s="78">
         <v>3</v>
       </c>
-      <c r="AJ1" s="64"/>
-      <c r="AK1" s="64"/>
-      <c r="AL1" s="64"/>
-      <c r="AM1" s="64"/>
-      <c r="AN1" s="66" t="s">
-        <v>36</v>
+      <c r="AJ1" s="63"/>
+      <c r="AK1" s="63"/>
+      <c r="AL1" s="63"/>
+      <c r="AM1" s="63"/>
+      <c r="AN1" s="64" t="s">
+        <v>1</v>
       </c>
       <c r="AO1" s="63"/>
       <c r="AP1" s="63"/>
@@ -1549,15 +1553,15 @@
       <c r="AR1" s="63"/>
       <c r="AS1" s="63"/>
       <c r="AT1" s="63"/>
-      <c r="AU1" s="64">
+      <c r="AU1" s="78">
         <v>4</v>
       </c>
-      <c r="AV1" s="64"/>
-      <c r="AW1" s="64"/>
-      <c r="AX1" s="64"/>
-      <c r="AY1" s="64"/>
-      <c r="AZ1" s="66" t="s">
-        <v>36</v>
+      <c r="AV1" s="63"/>
+      <c r="AW1" s="63"/>
+      <c r="AX1" s="63"/>
+      <c r="AY1" s="63"/>
+      <c r="AZ1" s="64" t="s">
+        <v>1</v>
       </c>
       <c r="BA1" s="63"/>
       <c r="BB1" s="63"/>
@@ -1565,263 +1569,263 @@
       <c r="BD1" s="63"/>
       <c r="BE1" s="63"/>
       <c r="BF1" s="63"/>
-      <c r="BG1" s="64">
+      <c r="BG1" s="89">
         <v>1</v>
       </c>
-      <c r="BH1" s="64"/>
-      <c r="BI1" s="64"/>
-      <c r="BJ1" s="64"/>
-      <c r="BK1" s="67"/>
+      <c r="BH1" s="63"/>
+      <c r="BI1" s="63"/>
+      <c r="BJ1" s="63"/>
+      <c r="BK1" s="90"/>
     </row>
     <row r="2" spans="1:64" x14ac:dyDescent="0.25">
-      <c r="C2" s="79"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="60" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="61" t="s">
-        <v>26</v>
-      </c>
-      <c r="I2" s="61"/>
-      <c r="J2" s="61"/>
-      <c r="K2" s="61"/>
-      <c r="L2" s="60"/>
-      <c r="M2" s="60"/>
-      <c r="N2" s="60"/>
-      <c r="O2" s="74"/>
-      <c r="P2" s="57"/>
-      <c r="Q2" s="60" t="s">
-        <v>25</v>
-      </c>
-      <c r="R2" s="60"/>
-      <c r="S2" s="60"/>
-      <c r="T2" s="61" t="s">
-        <v>27</v>
-      </c>
-      <c r="U2" s="61"/>
-      <c r="V2" s="61"/>
-      <c r="W2" s="61"/>
-      <c r="X2" s="60"/>
-      <c r="Y2" s="60"/>
-      <c r="Z2" s="60"/>
-      <c r="AA2" s="60"/>
-      <c r="AB2" s="58"/>
-      <c r="AC2" s="60" t="s">
-        <v>25</v>
-      </c>
-      <c r="AD2" s="60"/>
-      <c r="AE2" s="60"/>
-      <c r="AF2" s="61" t="s">
-        <v>28</v>
-      </c>
-      <c r="AG2" s="61"/>
-      <c r="AH2" s="61"/>
-      <c r="AI2" s="61"/>
-      <c r="AJ2" s="60"/>
-      <c r="AK2" s="60"/>
-      <c r="AL2" s="60"/>
-      <c r="AM2" s="60"/>
-      <c r="AN2" s="58"/>
-      <c r="AO2" s="60" t="s">
-        <v>25</v>
-      </c>
-      <c r="AP2" s="60"/>
-      <c r="AQ2" s="60"/>
-      <c r="AR2" s="61" t="s">
-        <v>29</v>
-      </c>
-      <c r="AS2" s="61"/>
-      <c r="AT2" s="61"/>
-      <c r="AU2" s="61"/>
-      <c r="AV2" s="60"/>
-      <c r="AW2" s="60"/>
-      <c r="AX2" s="60"/>
-      <c r="AY2" s="60"/>
-      <c r="AZ2" s="58"/>
-      <c r="BA2" s="60" t="s">
-        <v>25</v>
-      </c>
-      <c r="BB2" s="60"/>
-      <c r="BC2" s="60"/>
-      <c r="BD2" s="61" t="s">
-        <v>30</v>
-      </c>
-      <c r="BE2" s="61"/>
-      <c r="BF2" s="61"/>
-      <c r="BG2" s="61"/>
-      <c r="BH2" s="60"/>
-      <c r="BI2" s="60"/>
-      <c r="BJ2" s="60"/>
-      <c r="BK2" s="60"/>
-      <c r="BL2" s="53"/>
+      <c r="C2" s="84"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="61" t="s">
+        <v>2</v>
+      </c>
+      <c r="F2" s="53"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="77" t="s">
+        <v>3</v>
+      </c>
+      <c r="I2" s="53"/>
+      <c r="J2" s="53"/>
+      <c r="K2" s="53"/>
+      <c r="L2" s="71"/>
+      <c r="M2" s="53"/>
+      <c r="N2" s="53"/>
+      <c r="O2" s="55"/>
+      <c r="P2" s="48"/>
+      <c r="Q2" s="61" t="s">
+        <v>2</v>
+      </c>
+      <c r="R2" s="53"/>
+      <c r="S2" s="53"/>
+      <c r="T2" s="77" t="s">
+        <v>4</v>
+      </c>
+      <c r="U2" s="53"/>
+      <c r="V2" s="53"/>
+      <c r="W2" s="53"/>
+      <c r="X2" s="61"/>
+      <c r="Y2" s="53"/>
+      <c r="Z2" s="53"/>
+      <c r="AA2" s="53"/>
+      <c r="AB2" s="49"/>
+      <c r="AC2" s="61" t="s">
+        <v>2</v>
+      </c>
+      <c r="AD2" s="53"/>
+      <c r="AE2" s="53"/>
+      <c r="AF2" s="77" t="s">
+        <v>5</v>
+      </c>
+      <c r="AG2" s="53"/>
+      <c r="AH2" s="53"/>
+      <c r="AI2" s="53"/>
+      <c r="AJ2" s="61"/>
+      <c r="AK2" s="53"/>
+      <c r="AL2" s="53"/>
+      <c r="AM2" s="53"/>
+      <c r="AN2" s="49"/>
+      <c r="AO2" s="61" t="s">
+        <v>2</v>
+      </c>
+      <c r="AP2" s="53"/>
+      <c r="AQ2" s="53"/>
+      <c r="AR2" s="77" t="s">
+        <v>6</v>
+      </c>
+      <c r="AS2" s="53"/>
+      <c r="AT2" s="53"/>
+      <c r="AU2" s="53"/>
+      <c r="AV2" s="61"/>
+      <c r="AW2" s="53"/>
+      <c r="AX2" s="53"/>
+      <c r="AY2" s="53"/>
+      <c r="AZ2" s="49"/>
+      <c r="BA2" s="61" t="s">
+        <v>2</v>
+      </c>
+      <c r="BB2" s="53"/>
+      <c r="BC2" s="53"/>
+      <c r="BD2" s="77" t="s">
+        <v>7</v>
+      </c>
+      <c r="BE2" s="53"/>
+      <c r="BF2" s="53"/>
+      <c r="BG2" s="53"/>
+      <c r="BH2" s="61"/>
+      <c r="BI2" s="53"/>
+      <c r="BJ2" s="53"/>
+      <c r="BK2" s="93"/>
+      <c r="BL2" s="44"/>
     </row>
     <row r="3" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="79"/>
-      <c r="D3" s="81" t="s">
-        <v>22</v>
-      </c>
-      <c r="E3" s="76"/>
-      <c r="F3" s="72"/>
-      <c r="G3" s="73"/>
-      <c r="H3" s="70"/>
-      <c r="I3" s="71"/>
-      <c r="J3" s="75" t="s">
-        <v>17</v>
-      </c>
-      <c r="K3" s="76"/>
-      <c r="L3" s="72"/>
-      <c r="M3" s="73"/>
-      <c r="N3" s="70"/>
-      <c r="O3" s="71"/>
-      <c r="P3" s="75" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q3" s="76"/>
-      <c r="R3" s="72"/>
-      <c r="S3" s="73"/>
-      <c r="T3" s="70"/>
-      <c r="U3" s="71"/>
-      <c r="V3" s="75" t="s">
-        <v>17</v>
-      </c>
-      <c r="W3" s="76"/>
-      <c r="X3" s="72"/>
-      <c r="Y3" s="73"/>
-      <c r="Z3" s="70"/>
-      <c r="AA3" s="71"/>
-      <c r="AB3" s="77" t="s">
-        <v>22</v>
-      </c>
-      <c r="AC3" s="76"/>
-      <c r="AD3" s="72"/>
-      <c r="AE3" s="73"/>
-      <c r="AF3" s="70"/>
-      <c r="AG3" s="71"/>
-      <c r="AH3" s="75" t="s">
-        <v>17</v>
-      </c>
-      <c r="AI3" s="76"/>
-      <c r="AJ3" s="72"/>
-      <c r="AK3" s="73"/>
-      <c r="AL3" s="70"/>
-      <c r="AM3" s="71"/>
-      <c r="AN3" s="75" t="s">
-        <v>22</v>
-      </c>
-      <c r="AO3" s="76"/>
-      <c r="AP3" s="72"/>
-      <c r="AQ3" s="73"/>
-      <c r="AR3" s="70"/>
-      <c r="AS3" s="71"/>
-      <c r="AT3" s="75" t="s">
-        <v>17</v>
-      </c>
-      <c r="AU3" s="76"/>
-      <c r="AV3" s="72"/>
-      <c r="AW3" s="73"/>
-      <c r="AX3" s="70"/>
-      <c r="AY3" s="71"/>
-      <c r="AZ3" s="75" t="s">
-        <v>22</v>
-      </c>
-      <c r="BA3" s="76"/>
-      <c r="BB3" s="72"/>
-      <c r="BC3" s="73"/>
-      <c r="BD3" s="70"/>
-      <c r="BE3" s="71"/>
-      <c r="BF3" s="75" t="s">
-        <v>17</v>
-      </c>
-      <c r="BG3" s="76"/>
-      <c r="BH3" s="72"/>
-      <c r="BI3" s="73"/>
-      <c r="BJ3" s="70"/>
-      <c r="BK3" s="70"/>
-      <c r="BL3" s="53"/>
-    </row>
-    <row r="4" spans="1:64" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="97"/>
-      <c r="C4" s="80"/>
+        <v>8</v>
+      </c>
+      <c r="C3" s="84"/>
+      <c r="D3" s="82" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="55"/>
+      <c r="F3" s="52"/>
+      <c r="G3" s="53"/>
+      <c r="H3" s="60"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="54" t="s">
+        <v>10</v>
+      </c>
+      <c r="K3" s="55"/>
+      <c r="L3" s="52"/>
+      <c r="M3" s="53"/>
+      <c r="N3" s="60"/>
+      <c r="O3" s="55"/>
+      <c r="P3" s="54" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q3" s="55"/>
+      <c r="R3" s="52"/>
+      <c r="S3" s="53"/>
+      <c r="T3" s="60"/>
+      <c r="U3" s="55"/>
+      <c r="V3" s="54" t="s">
+        <v>10</v>
+      </c>
+      <c r="W3" s="55"/>
+      <c r="X3" s="52"/>
+      <c r="Y3" s="53"/>
+      <c r="Z3" s="60"/>
+      <c r="AA3" s="55"/>
+      <c r="AB3" s="92" t="s">
+        <v>9</v>
+      </c>
+      <c r="AC3" s="55"/>
+      <c r="AD3" s="52"/>
+      <c r="AE3" s="53"/>
+      <c r="AF3" s="60"/>
+      <c r="AG3" s="55"/>
+      <c r="AH3" s="54" t="s">
+        <v>10</v>
+      </c>
+      <c r="AI3" s="55"/>
+      <c r="AJ3" s="52"/>
+      <c r="AK3" s="53"/>
+      <c r="AL3" s="60"/>
+      <c r="AM3" s="55"/>
+      <c r="AN3" s="54" t="s">
+        <v>9</v>
+      </c>
+      <c r="AO3" s="55"/>
+      <c r="AP3" s="52"/>
+      <c r="AQ3" s="53"/>
+      <c r="AR3" s="60"/>
+      <c r="AS3" s="55"/>
+      <c r="AT3" s="54" t="s">
+        <v>10</v>
+      </c>
+      <c r="AU3" s="55"/>
+      <c r="AV3" s="52"/>
+      <c r="AW3" s="53"/>
+      <c r="AX3" s="60"/>
+      <c r="AY3" s="55"/>
+      <c r="AZ3" s="54" t="s">
+        <v>9</v>
+      </c>
+      <c r="BA3" s="55"/>
+      <c r="BB3" s="52"/>
+      <c r="BC3" s="53"/>
+      <c r="BD3" s="60"/>
+      <c r="BE3" s="55"/>
+      <c r="BF3" s="54" t="s">
+        <v>10</v>
+      </c>
+      <c r="BG3" s="55"/>
+      <c r="BH3" s="52"/>
+      <c r="BI3" s="53"/>
+      <c r="BJ3" s="76"/>
+      <c r="BK3" s="93"/>
+      <c r="BL3" s="44"/>
+    </row>
+    <row r="4" spans="1:64" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="51"/>
+      <c r="C4" s="85"/>
       <c r="D4" s="88" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" s="89"/>
-      <c r="F4" s="90"/>
+        <v>11</v>
+      </c>
+      <c r="E4" s="66"/>
+      <c r="F4" s="67"/>
       <c r="G4" s="91" t="s">
-        <v>37</v>
-      </c>
-      <c r="H4" s="92"/>
-      <c r="I4" s="92"/>
-      <c r="J4" s="92"/>
-      <c r="K4" s="92"/>
-      <c r="L4" s="92"/>
-      <c r="M4" s="92"/>
-      <c r="N4" s="92"/>
-      <c r="O4" s="92"/>
-      <c r="P4" s="93" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q4" s="89"/>
-      <c r="R4" s="90"/>
-      <c r="S4" s="91"/>
-      <c r="T4" s="92"/>
-      <c r="U4" s="92"/>
-      <c r="V4" s="92"/>
-      <c r="W4" s="92"/>
-      <c r="X4" s="92"/>
-      <c r="Y4" s="92"/>
-      <c r="Z4" s="92"/>
-      <c r="AA4" s="94"/>
-      <c r="AB4" s="93" t="s">
-        <v>23</v>
-      </c>
-      <c r="AC4" s="89"/>
-      <c r="AD4" s="90"/>
-      <c r="AE4" s="91"/>
-      <c r="AF4" s="92"/>
-      <c r="AG4" s="92"/>
-      <c r="AH4" s="92"/>
-      <c r="AI4" s="92"/>
-      <c r="AJ4" s="92"/>
-      <c r="AK4" s="92"/>
-      <c r="AL4" s="92"/>
-      <c r="AM4" s="92"/>
-      <c r="AN4" s="93" t="s">
-        <v>23</v>
-      </c>
-      <c r="AO4" s="89"/>
-      <c r="AP4" s="90"/>
-      <c r="AQ4" s="91"/>
-      <c r="AR4" s="92"/>
-      <c r="AS4" s="92"/>
-      <c r="AT4" s="92"/>
-      <c r="AU4" s="92"/>
-      <c r="AV4" s="92"/>
-      <c r="AW4" s="92"/>
-      <c r="AX4" s="92"/>
-      <c r="AY4" s="92"/>
-      <c r="AZ4" s="93" t="s">
-        <v>23</v>
-      </c>
-      <c r="BA4" s="89"/>
-      <c r="BB4" s="90"/>
-      <c r="BC4" s="91"/>
-      <c r="BD4" s="92"/>
-      <c r="BE4" s="92"/>
-      <c r="BF4" s="92"/>
-      <c r="BG4" s="92"/>
-      <c r="BH4" s="92"/>
-      <c r="BI4" s="92"/>
-      <c r="BJ4" s="92"/>
-      <c r="BK4" s="96"/>
+        <v>12</v>
+      </c>
+      <c r="H4" s="66"/>
+      <c r="I4" s="66"/>
+      <c r="J4" s="66"/>
+      <c r="K4" s="66"/>
+      <c r="L4" s="66"/>
+      <c r="M4" s="66"/>
+      <c r="N4" s="66"/>
+      <c r="O4" s="66"/>
+      <c r="P4" s="68" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q4" s="66"/>
+      <c r="R4" s="67"/>
+      <c r="S4" s="65"/>
+      <c r="T4" s="66"/>
+      <c r="U4" s="66"/>
+      <c r="V4" s="66"/>
+      <c r="W4" s="66"/>
+      <c r="X4" s="66"/>
+      <c r="Y4" s="66"/>
+      <c r="Z4" s="66"/>
+      <c r="AA4" s="67"/>
+      <c r="AB4" s="68" t="s">
+        <v>11</v>
+      </c>
+      <c r="AC4" s="66"/>
+      <c r="AD4" s="67"/>
+      <c r="AE4" s="79"/>
+      <c r="AF4" s="66"/>
+      <c r="AG4" s="66"/>
+      <c r="AH4" s="66"/>
+      <c r="AI4" s="66"/>
+      <c r="AJ4" s="66"/>
+      <c r="AK4" s="66"/>
+      <c r="AL4" s="66"/>
+      <c r="AM4" s="66"/>
+      <c r="AN4" s="68" t="s">
+        <v>11</v>
+      </c>
+      <c r="AO4" s="66"/>
+      <c r="AP4" s="67"/>
+      <c r="AQ4" s="79"/>
+      <c r="AR4" s="66"/>
+      <c r="AS4" s="66"/>
+      <c r="AT4" s="66"/>
+      <c r="AU4" s="66"/>
+      <c r="AV4" s="66"/>
+      <c r="AW4" s="66"/>
+      <c r="AX4" s="66"/>
+      <c r="AY4" s="66"/>
+      <c r="AZ4" s="68" t="s">
+        <v>11</v>
+      </c>
+      <c r="BA4" s="66"/>
+      <c r="BB4" s="67"/>
+      <c r="BC4" s="80"/>
+      <c r="BD4" s="66"/>
+      <c r="BE4" s="66"/>
+      <c r="BF4" s="66"/>
+      <c r="BG4" s="66"/>
+      <c r="BH4" s="66"/>
+      <c r="BI4" s="66"/>
+      <c r="BJ4" s="66"/>
+      <c r="BK4" s="81"/>
     </row>
     <row r="5" spans="1:64" ht="20.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="59"/>
+      <c r="B5" s="50"/>
       <c r="C5" s="2"/>
       <c r="D5" s="11">
         <v>1</v>
@@ -1836,25 +1840,25 @@
         <v>4</v>
       </c>
       <c r="H5" s="12" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="I5" s="12">
         <v>5</v>
       </c>
       <c r="J5" s="12" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="K5" s="12">
         <v>6</v>
       </c>
       <c r="L5" s="12" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="M5" s="12">
         <v>7</v>
       </c>
       <c r="N5" s="12" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="O5" s="13">
         <v>8</v>
@@ -1872,25 +1876,25 @@
         <v>4</v>
       </c>
       <c r="T5" s="12" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="U5" s="12">
         <v>5</v>
       </c>
       <c r="V5" s="12" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="W5" s="12">
         <v>6</v>
       </c>
       <c r="X5" s="12" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="Y5" s="12">
         <v>7</v>
       </c>
       <c r="Z5" s="12" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="AA5" s="13">
         <v>8</v>
@@ -1908,25 +1912,25 @@
         <v>4</v>
       </c>
       <c r="AF5" s="12" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="AG5" s="12">
         <v>5</v>
       </c>
       <c r="AH5" s="12" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="AI5" s="12">
         <v>6</v>
       </c>
       <c r="AJ5" s="12" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="AK5" s="12">
         <v>7</v>
       </c>
       <c r="AL5" s="12" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="AM5" s="13">
         <v>8</v>
@@ -1944,25 +1948,25 @@
         <v>4</v>
       </c>
       <c r="AR5" s="12" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="AS5" s="12">
         <v>5</v>
       </c>
       <c r="AT5" s="12" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="AU5" s="12">
         <v>6</v>
       </c>
       <c r="AV5" s="12" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="AW5" s="12">
         <v>7</v>
       </c>
       <c r="AX5" s="12" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="AY5" s="13">
         <v>8</v>
@@ -1980,25 +1984,25 @@
         <v>4</v>
       </c>
       <c r="BD5" s="12" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="BE5" s="12">
         <v>5</v>
       </c>
       <c r="BF5" s="12" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="BG5" s="12">
         <v>6</v>
       </c>
       <c r="BH5" s="12" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="BI5" s="12">
         <v>7</v>
       </c>
       <c r="BJ5" s="12" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="BK5" s="14">
         <v>8</v>
@@ -2009,7 +2013,7 @@
         <v>1</v>
       </c>
       <c r="C6" s="28" t="s">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="D6" s="31"/>
       <c r="E6" s="18"/>
@@ -3198,6 +3202,7 @@
       <c r="B24" s="26">
         <v>19</v>
       </c>
+      <c r="C24"/>
       <c r="D24" s="31"/>
       <c r="E24" s="18"/>
       <c r="F24" s="32"/>
@@ -3210,120 +3215,120 @@
       <c r="M24" s="32"/>
       <c r="N24" s="36"/>
       <c r="O24" s="36"/>
-      <c r="P24" s="44"/>
-      <c r="Q24" s="45"/>
-      <c r="R24" s="46"/>
-      <c r="S24" s="47"/>
-      <c r="T24" s="48"/>
-      <c r="U24" s="49"/>
-      <c r="V24" s="45"/>
-      <c r="W24" s="50"/>
-      <c r="X24" s="46"/>
-      <c r="Y24" s="46"/>
-      <c r="Z24" s="51"/>
-      <c r="AA24" s="51"/>
-      <c r="AB24" s="44"/>
-      <c r="AC24" s="45"/>
-      <c r="AD24" s="46"/>
-      <c r="AE24" s="47"/>
-      <c r="AF24" s="48"/>
-      <c r="AG24" s="49"/>
-      <c r="AH24" s="45"/>
-      <c r="AI24" s="50"/>
-      <c r="AJ24" s="46"/>
-      <c r="AK24" s="46"/>
-      <c r="AL24" s="51"/>
-      <c r="AM24" s="51"/>
-      <c r="AN24" s="44"/>
-      <c r="AO24" s="45"/>
-      <c r="AP24" s="46"/>
-      <c r="AQ24" s="47"/>
-      <c r="AR24" s="48"/>
-      <c r="AS24" s="49"/>
-      <c r="AT24" s="45"/>
-      <c r="AU24" s="50"/>
-      <c r="AV24" s="46"/>
-      <c r="AW24" s="46"/>
-      <c r="AX24" s="51"/>
-      <c r="AY24" s="51"/>
-      <c r="AZ24" s="44"/>
-      <c r="BA24" s="45"/>
-      <c r="BB24" s="46"/>
-      <c r="BC24" s="47"/>
-      <c r="BD24" s="48"/>
-      <c r="BE24" s="49"/>
-      <c r="BF24" s="45"/>
-      <c r="BG24" s="50"/>
-      <c r="BH24" s="46"/>
-      <c r="BI24" s="46"/>
-      <c r="BJ24" s="51"/>
-      <c r="BK24" s="52"/>
-    </row>
-    <row r="25" spans="2:64" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="P24" s="31"/>
+      <c r="Q24" s="18"/>
+      <c r="R24" s="32"/>
+      <c r="S24" s="33"/>
+      <c r="T24" s="34"/>
+      <c r="U24" s="35"/>
+      <c r="V24" s="18"/>
+      <c r="W24" s="19"/>
+      <c r="X24" s="32"/>
+      <c r="Y24" s="32"/>
+      <c r="Z24" s="36"/>
+      <c r="AA24" s="36"/>
+      <c r="AB24" s="31"/>
+      <c r="AC24" s="18"/>
+      <c r="AD24" s="32"/>
+      <c r="AE24" s="33"/>
+      <c r="AF24" s="34"/>
+      <c r="AG24" s="35"/>
+      <c r="AH24" s="18"/>
+      <c r="AI24" s="19"/>
+      <c r="AJ24" s="32"/>
+      <c r="AK24" s="32"/>
+      <c r="AL24" s="36"/>
+      <c r="AM24" s="36"/>
+      <c r="AN24" s="31"/>
+      <c r="AO24" s="18"/>
+      <c r="AP24" s="32"/>
+      <c r="AQ24" s="33"/>
+      <c r="AR24" s="34"/>
+      <c r="AS24" s="35"/>
+      <c r="AT24" s="18"/>
+      <c r="AU24" s="19"/>
+      <c r="AV24" s="32"/>
+      <c r="AW24" s="32"/>
+      <c r="AX24" s="36"/>
+      <c r="AY24" s="36"/>
+      <c r="AZ24" s="31"/>
+      <c r="BA24" s="18"/>
+      <c r="BB24" s="32"/>
+      <c r="BC24" s="33"/>
+      <c r="BD24" s="34"/>
+      <c r="BE24" s="35"/>
+      <c r="BF24" s="18"/>
+      <c r="BG24" s="19"/>
+      <c r="BH24" s="32"/>
+      <c r="BI24" s="32"/>
+      <c r="BJ24" s="36"/>
+      <c r="BK24" s="37"/>
+    </row>
+    <row r="25" spans="2:64" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C25" s="42" t="s">
-        <v>21</v>
-      </c>
-      <c r="D25" s="82" t="s">
         <v>18</v>
       </c>
-      <c r="E25" s="83"/>
-      <c r="F25" s="83"/>
-      <c r="G25" s="83"/>
-      <c r="H25" s="83"/>
-      <c r="I25" s="83"/>
-      <c r="J25" s="83"/>
-      <c r="K25" s="83"/>
-      <c r="L25" s="83"/>
-      <c r="M25" s="83"/>
-      <c r="N25" s="83"/>
-      <c r="O25" s="84"/>
+      <c r="D25" s="73" t="s">
+        <v>19</v>
+      </c>
+      <c r="E25" s="74"/>
+      <c r="F25" s="74"/>
+      <c r="G25" s="74"/>
+      <c r="H25" s="74"/>
+      <c r="I25" s="74"/>
+      <c r="J25" s="74"/>
+      <c r="K25" s="74"/>
+      <c r="L25" s="74"/>
+      <c r="M25" s="74"/>
+      <c r="N25" s="74"/>
+      <c r="O25" s="75"/>
       <c r="AB25" s="7"/>
       <c r="AM25" s="8"/>
-      <c r="AN25" s="85" t="s">
+      <c r="AN25" s="56" t="s">
+        <v>20</v>
+      </c>
+      <c r="AO25" s="57"/>
+      <c r="AP25" s="57"/>
+      <c r="AQ25" s="57"/>
+      <c r="AR25" s="57"/>
+      <c r="AS25" s="57"/>
+      <c r="AT25" s="57"/>
+      <c r="AU25" s="57"/>
+      <c r="AV25" s="57"/>
+      <c r="AW25" s="57"/>
+      <c r="AX25" s="57"/>
+      <c r="AY25" s="58"/>
+      <c r="AZ25" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="AO25" s="86"/>
-      <c r="AP25" s="86"/>
-      <c r="AQ25" s="86"/>
-      <c r="AR25" s="86"/>
-      <c r="AS25" s="86"/>
-      <c r="AT25" s="86"/>
-      <c r="AU25" s="86"/>
-      <c r="AV25" s="86"/>
-      <c r="AW25" s="86"/>
-      <c r="AX25" s="86"/>
-      <c r="AY25" s="87"/>
-      <c r="AZ25" s="85" t="s">
-        <v>18</v>
-      </c>
-      <c r="BA25" s="86"/>
-      <c r="BB25" s="86"/>
-      <c r="BC25" s="86"/>
-      <c r="BD25" s="86"/>
-      <c r="BE25" s="86"/>
-      <c r="BF25" s="86"/>
-      <c r="BG25" s="86"/>
-      <c r="BH25" s="86"/>
-      <c r="BI25" s="86"/>
-      <c r="BJ25" s="86"/>
-      <c r="BK25" s="86"/>
-      <c r="BL25" s="53"/>
+      <c r="BA25" s="57"/>
+      <c r="BB25" s="57"/>
+      <c r="BC25" s="57"/>
+      <c r="BD25" s="57"/>
+      <c r="BE25" s="57"/>
+      <c r="BF25" s="57"/>
+      <c r="BG25" s="57"/>
+      <c r="BH25" s="57"/>
+      <c r="BI25" s="57"/>
+      <c r="BJ25" s="57"/>
+      <c r="BK25" s="57"/>
+      <c r="BL25" s="44"/>
     </row>
     <row r="26" spans="2:64" x14ac:dyDescent="0.25">
-      <c r="C26" s="54" t="s">
-        <v>24</v>
-      </c>
-      <c r="D26" s="68"/>
-      <c r="E26" s="69"/>
+      <c r="C26" s="45" t="s">
+        <v>21</v>
+      </c>
+      <c r="D26" s="69"/>
+      <c r="E26" s="55"/>
       <c r="F26" s="3"/>
       <c r="O26" s="8"/>
-      <c r="P26" s="68"/>
-      <c r="Q26" s="69"/>
-      <c r="AB26" s="68"/>
-      <c r="AC26" s="69"/>
+      <c r="P26" s="69"/>
+      <c r="Q26" s="55"/>
+      <c r="AB26" s="69"/>
+      <c r="AC26" s="55"/>
       <c r="AM26" s="8"/>
-      <c r="AN26" s="68"/>
-      <c r="AO26" s="69"/>
+      <c r="AN26" s="69"/>
+      <c r="AO26" s="55"/>
       <c r="AP26" s="21"/>
       <c r="AQ26" s="21"/>
       <c r="AR26" s="21"/>
@@ -3334,28 +3339,28 @@
       <c r="AW26" s="21"/>
       <c r="AX26" s="21"/>
       <c r="AY26" s="30"/>
-      <c r="AZ26" s="68"/>
-      <c r="BA26" s="69"/>
+      <c r="AZ26" s="69"/>
+      <c r="BA26" s="55"/>
       <c r="BK26" s="5"/>
     </row>
     <row r="27" spans="2:64" x14ac:dyDescent="0.25">
       <c r="C27" s="38" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="D27" s="17"/>
-      <c r="E27" s="55" t="s">
-        <v>12</v>
-      </c>
-      <c r="G27" s="95" t="s">
-        <v>20</v>
-      </c>
-      <c r="H27" s="95"/>
-      <c r="I27" s="95"/>
-      <c r="J27" s="95"/>
-      <c r="K27" s="95"/>
-      <c r="L27" s="95"/>
-      <c r="M27" s="95"/>
-      <c r="N27" s="95"/>
+      <c r="E27" s="46" t="s">
+        <v>23</v>
+      </c>
+      <c r="G27" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="H27" s="57"/>
+      <c r="I27" s="57"/>
+      <c r="J27" s="57"/>
+      <c r="K27" s="57"/>
+      <c r="L27" s="57"/>
+      <c r="M27" s="57"/>
+      <c r="N27" s="57"/>
       <c r="O27" s="8"/>
       <c r="P27" s="1"/>
       <c r="Q27" s="3"/>
@@ -3365,39 +3370,39 @@
       <c r="AM27" s="8"/>
       <c r="AN27" s="17"/>
       <c r="AO27" s="23" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="AP27" s="21"/>
-      <c r="AQ27" s="95" t="s">
-        <v>20</v>
-      </c>
-      <c r="AR27" s="95"/>
-      <c r="AS27" s="95"/>
-      <c r="AT27" s="95"/>
-      <c r="AU27" s="95"/>
-      <c r="AV27" s="95"/>
-      <c r="AW27" s="95"/>
-      <c r="AX27" s="95"/>
+      <c r="AQ27" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="AR27" s="57"/>
+      <c r="AS27" s="57"/>
+      <c r="AT27" s="57"/>
+      <c r="AU27" s="57"/>
+      <c r="AV27" s="57"/>
+      <c r="AW27" s="57"/>
+      <c r="AX27" s="57"/>
       <c r="AY27" s="43"/>
       <c r="AZ27" s="17"/>
       <c r="BA27" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="BC27" s="95" t="s">
-        <v>20</v>
-      </c>
-      <c r="BD27" s="95"/>
-      <c r="BE27" s="95"/>
-      <c r="BF27" s="95"/>
-      <c r="BG27" s="95"/>
-      <c r="BH27" s="95"/>
-      <c r="BI27" s="95"/>
-      <c r="BJ27" s="95"/>
+        <v>23</v>
+      </c>
+      <c r="BC27" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="BD27" s="57"/>
+      <c r="BE27" s="57"/>
+      <c r="BF27" s="57"/>
+      <c r="BG27" s="57"/>
+      <c r="BH27" s="57"/>
+      <c r="BI27" s="57"/>
+      <c r="BJ27" s="57"/>
       <c r="BK27" s="5"/>
     </row>
     <row r="28" spans="2:64" x14ac:dyDescent="0.25">
       <c r="C28" s="38" t="s">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="D28" s="15"/>
       <c r="E28" s="3"/>
@@ -3416,11 +3421,11 @@
     </row>
     <row r="29" spans="2:64" x14ac:dyDescent="0.25">
       <c r="C29" s="38" t="s">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="D29" s="1"/>
       <c r="E29" s="22" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="O29" s="8"/>
       <c r="P29" s="1"/>
@@ -3431,17 +3436,17 @@
       <c r="AM29" s="8"/>
       <c r="AN29" s="1"/>
       <c r="AO29" s="22" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="AZ29" s="1"/>
       <c r="BA29" s="22" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="BK29" s="5"/>
     </row>
     <row r="30" spans="2:64" x14ac:dyDescent="0.25">
       <c r="C30" s="38" t="s">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="D30" s="1"/>
       <c r="E30" s="3"/>
@@ -3458,9 +3463,9 @@
       <c r="BA30" s="3"/>
       <c r="BK30" s="5"/>
     </row>
-    <row r="31" spans="2:64" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:64" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C31" s="39" t="s">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="D31" s="16"/>
       <c r="E31" s="10"/>
@@ -3523,86 +3528,86 @@
       <c r="BJ31" s="4"/>
       <c r="BK31" s="6"/>
     </row>
-    <row r="32" spans="2:64" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="2:64" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="77">
-    <mergeCell ref="G27:N27"/>
-    <mergeCell ref="AQ27:AX27"/>
-    <mergeCell ref="BC27:BJ27"/>
-    <mergeCell ref="AE4:AM4"/>
-    <mergeCell ref="AN4:AP4"/>
-    <mergeCell ref="AQ4:AY4"/>
+    <mergeCell ref="C1:C4"/>
     <mergeCell ref="AZ4:BB4"/>
-    <mergeCell ref="BC4:BK4"/>
-    <mergeCell ref="BJ3:BK3"/>
-    <mergeCell ref="AR2:AU2"/>
-    <mergeCell ref="D25:O25"/>
-    <mergeCell ref="AN25:AY25"/>
-    <mergeCell ref="AZ25:BK25"/>
-    <mergeCell ref="AZ3:BA3"/>
+    <mergeCell ref="F3:G3"/>
     <mergeCell ref="BF3:BG3"/>
+    <mergeCell ref="BH3:BI3"/>
+    <mergeCell ref="K1:O1"/>
     <mergeCell ref="D4:F4"/>
+    <mergeCell ref="W1:AA1"/>
+    <mergeCell ref="BG1:BK1"/>
     <mergeCell ref="G4:O4"/>
-    <mergeCell ref="P4:R4"/>
-    <mergeCell ref="S4:AA4"/>
-    <mergeCell ref="AB4:AD4"/>
-    <mergeCell ref="AH3:AI3"/>
-    <mergeCell ref="AV3:AW3"/>
-    <mergeCell ref="AX3:AY3"/>
-    <mergeCell ref="BB3:BC3"/>
-    <mergeCell ref="BD3:BE3"/>
-    <mergeCell ref="BH3:BI3"/>
-    <mergeCell ref="P3:Q3"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="N3:O3"/>
-    <mergeCell ref="AN3:AO3"/>
-    <mergeCell ref="AT3:AU3"/>
-    <mergeCell ref="C1:C4"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="AF2:AI2"/>
-    <mergeCell ref="AJ2:AM2"/>
-    <mergeCell ref="AO2:AQ2"/>
-    <mergeCell ref="V3:W3"/>
-    <mergeCell ref="AB3:AC3"/>
-    <mergeCell ref="L2:O2"/>
     <mergeCell ref="Q2:S2"/>
-    <mergeCell ref="T2:W2"/>
-    <mergeCell ref="X2:AA2"/>
     <mergeCell ref="AC2:AE2"/>
     <mergeCell ref="R3:S3"/>
-    <mergeCell ref="T3:U3"/>
+    <mergeCell ref="AE4:AM4"/>
+    <mergeCell ref="BA2:BC2"/>
+    <mergeCell ref="AR3:AS3"/>
+    <mergeCell ref="D1:J1"/>
     <mergeCell ref="X3:Y3"/>
+    <mergeCell ref="D25:O25"/>
     <mergeCell ref="Z3:AA3"/>
-    <mergeCell ref="AD3:AE3"/>
-    <mergeCell ref="AF3:AG3"/>
     <mergeCell ref="AJ3:AK3"/>
-    <mergeCell ref="AL3:AM3"/>
-    <mergeCell ref="AP3:AQ3"/>
-    <mergeCell ref="AR3:AS3"/>
+    <mergeCell ref="AB1:AH1"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="T2:W2"/>
+    <mergeCell ref="AB4:AD4"/>
+    <mergeCell ref="AF2:AI2"/>
+    <mergeCell ref="AI1:AM1"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="P3:Q3"/>
+    <mergeCell ref="H2:K2"/>
     <mergeCell ref="D26:E26"/>
     <mergeCell ref="P26:Q26"/>
+    <mergeCell ref="G27:N27"/>
+    <mergeCell ref="AZ25:BK25"/>
+    <mergeCell ref="L2:O2"/>
+    <mergeCell ref="AL3:AM3"/>
+    <mergeCell ref="AV2:AY2"/>
+    <mergeCell ref="BH2:BK2"/>
+    <mergeCell ref="BJ3:BK3"/>
+    <mergeCell ref="AN4:AP4"/>
     <mergeCell ref="AB26:AC26"/>
     <mergeCell ref="AN26:AO26"/>
-    <mergeCell ref="AZ26:BA26"/>
-    <mergeCell ref="AV2:AY2"/>
-    <mergeCell ref="BA2:BC2"/>
+    <mergeCell ref="AQ4:AY4"/>
+    <mergeCell ref="BC4:BK4"/>
     <mergeCell ref="BD2:BG2"/>
-    <mergeCell ref="BH2:BK2"/>
-    <mergeCell ref="D1:J1"/>
-    <mergeCell ref="K1:O1"/>
+    <mergeCell ref="AX3:AY3"/>
     <mergeCell ref="P1:V1"/>
-    <mergeCell ref="W1:AA1"/>
-    <mergeCell ref="AB1:AH1"/>
-    <mergeCell ref="AI1:AM1"/>
+    <mergeCell ref="AZ1:BF1"/>
+    <mergeCell ref="AJ2:AM2"/>
+    <mergeCell ref="S4:AA4"/>
+    <mergeCell ref="P4:R4"/>
+    <mergeCell ref="AO2:AQ2"/>
     <mergeCell ref="AN1:AT1"/>
     <mergeCell ref="AU1:AY1"/>
-    <mergeCell ref="AZ1:BF1"/>
-    <mergeCell ref="BG1:BK1"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="H2:K2"/>
+    <mergeCell ref="AZ3:BA3"/>
+    <mergeCell ref="T3:U3"/>
+    <mergeCell ref="V3:W3"/>
+    <mergeCell ref="AF3:AG3"/>
+    <mergeCell ref="AH3:AI3"/>
+    <mergeCell ref="BB3:BC3"/>
+    <mergeCell ref="AR2:AU2"/>
+    <mergeCell ref="AB3:AC3"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="AT3:AU3"/>
+    <mergeCell ref="AV3:AW3"/>
+    <mergeCell ref="N3:O3"/>
+    <mergeCell ref="X2:AA2"/>
+    <mergeCell ref="AD3:AE3"/>
+    <mergeCell ref="AN3:AO3"/>
+    <mergeCell ref="AP3:AQ3"/>
+    <mergeCell ref="AN25:AY25"/>
+    <mergeCell ref="BC27:BJ27"/>
+    <mergeCell ref="BD3:BE3"/>
+    <mergeCell ref="AQ27:AX27"/>
+    <mergeCell ref="AZ26:BA26"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0" footer="0"/>
@@ -3611,7 +3616,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6C3F5C7-FB5E-4E6D-ADE2-CC6EF23B61E1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:BL32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3621,11 +3626,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:64" ht="17.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="C1" s="78" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="62" t="s">
-        <v>36</v>
+      <c r="C1" s="83" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="72" t="s">
+        <v>1</v>
       </c>
       <c r="E1" s="63"/>
       <c r="F1" s="63"/>
@@ -3633,15 +3638,15 @@
       <c r="H1" s="63"/>
       <c r="I1" s="63"/>
       <c r="J1" s="63"/>
-      <c r="K1" s="64">
+      <c r="K1" s="86">
         <v>3</v>
       </c>
-      <c r="L1" s="64"/>
-      <c r="M1" s="64"/>
-      <c r="N1" s="64"/>
-      <c r="O1" s="65"/>
-      <c r="P1" s="63" t="s">
-        <v>36</v>
+      <c r="L1" s="63"/>
+      <c r="M1" s="63"/>
+      <c r="N1" s="63"/>
+      <c r="O1" s="87"/>
+      <c r="P1" s="62" t="s">
+        <v>1</v>
       </c>
       <c r="Q1" s="63"/>
       <c r="R1" s="63"/>
@@ -3649,15 +3654,15 @@
       <c r="T1" s="63"/>
       <c r="U1" s="63"/>
       <c r="V1" s="63"/>
-      <c r="W1" s="64">
+      <c r="W1" s="78">
         <v>4</v>
       </c>
-      <c r="X1" s="64"/>
-      <c r="Y1" s="64"/>
-      <c r="Z1" s="64"/>
-      <c r="AA1" s="64"/>
-      <c r="AB1" s="66" t="s">
-        <v>36</v>
+      <c r="X1" s="63"/>
+      <c r="Y1" s="63"/>
+      <c r="Z1" s="63"/>
+      <c r="AA1" s="63"/>
+      <c r="AB1" s="64" t="s">
+        <v>1</v>
       </c>
       <c r="AC1" s="63"/>
       <c r="AD1" s="63"/>
@@ -3665,15 +3670,15 @@
       <c r="AF1" s="63"/>
       <c r="AG1" s="63"/>
       <c r="AH1" s="63"/>
-      <c r="AI1" s="64">
+      <c r="AI1" s="78">
         <v>1</v>
       </c>
-      <c r="AJ1" s="64"/>
-      <c r="AK1" s="64"/>
-      <c r="AL1" s="64"/>
-      <c r="AM1" s="64"/>
-      <c r="AN1" s="66" t="s">
-        <v>36</v>
+      <c r="AJ1" s="63"/>
+      <c r="AK1" s="63"/>
+      <c r="AL1" s="63"/>
+      <c r="AM1" s="63"/>
+      <c r="AN1" s="64" t="s">
+        <v>1</v>
       </c>
       <c r="AO1" s="63"/>
       <c r="AP1" s="63"/>
@@ -3681,15 +3686,15 @@
       <c r="AR1" s="63"/>
       <c r="AS1" s="63"/>
       <c r="AT1" s="63"/>
-      <c r="AU1" s="64">
+      <c r="AU1" s="78">
         <v>2</v>
       </c>
-      <c r="AV1" s="64"/>
-      <c r="AW1" s="64"/>
-      <c r="AX1" s="64"/>
-      <c r="AY1" s="64"/>
-      <c r="AZ1" s="66" t="s">
-        <v>36</v>
+      <c r="AV1" s="63"/>
+      <c r="AW1" s="63"/>
+      <c r="AX1" s="63"/>
+      <c r="AY1" s="63"/>
+      <c r="AZ1" s="64" t="s">
+        <v>1</v>
       </c>
       <c r="BA1" s="63"/>
       <c r="BB1" s="63"/>
@@ -3697,260 +3702,261 @@
       <c r="BD1" s="63"/>
       <c r="BE1" s="63"/>
       <c r="BF1" s="63"/>
-      <c r="BG1" s="64">
+      <c r="BG1" s="89">
         <v>3</v>
       </c>
-      <c r="BH1" s="64"/>
-      <c r="BI1" s="64"/>
-      <c r="BJ1" s="64"/>
-      <c r="BK1" s="67"/>
+      <c r="BH1" s="63"/>
+      <c r="BI1" s="63"/>
+      <c r="BJ1" s="63"/>
+      <c r="BK1" s="90"/>
     </row>
     <row r="2" spans="1:64" x14ac:dyDescent="0.25">
-      <c r="C2" s="79"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="60" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="61" t="s">
-        <v>31</v>
-      </c>
-      <c r="I2" s="61"/>
-      <c r="J2" s="61"/>
-      <c r="K2" s="61"/>
-      <c r="L2" s="60"/>
-      <c r="M2" s="60"/>
-      <c r="N2" s="60"/>
-      <c r="O2" s="74"/>
-      <c r="P2" s="57"/>
-      <c r="Q2" s="60" t="s">
-        <v>25</v>
-      </c>
-      <c r="R2" s="60"/>
-      <c r="S2" s="60"/>
-      <c r="T2" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="U2" s="61"/>
-      <c r="V2" s="61"/>
-      <c r="W2" s="61"/>
-      <c r="X2" s="60"/>
-      <c r="Y2" s="60"/>
-      <c r="Z2" s="60"/>
-      <c r="AA2" s="60"/>
-      <c r="AB2" s="58"/>
-      <c r="AC2" s="60" t="s">
-        <v>25</v>
-      </c>
-      <c r="AD2" s="60"/>
-      <c r="AE2" s="60"/>
-      <c r="AF2" s="61" t="s">
+      <c r="C2" s="84"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="61" t="s">
+        <v>2</v>
+      </c>
+      <c r="F2" s="53"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="77" t="s">
         <v>33</v>
       </c>
-      <c r="AG2" s="61"/>
-      <c r="AH2" s="61"/>
-      <c r="AI2" s="61"/>
-      <c r="AJ2" s="60"/>
-      <c r="AK2" s="60"/>
-      <c r="AL2" s="60"/>
-      <c r="AM2" s="60"/>
-      <c r="AN2" s="58"/>
-      <c r="AO2" s="60" t="s">
-        <v>25</v>
-      </c>
-      <c r="AP2" s="60"/>
-      <c r="AQ2" s="60"/>
-      <c r="AR2" s="61" t="s">
+      <c r="I2" s="53"/>
+      <c r="J2" s="53"/>
+      <c r="K2" s="53"/>
+      <c r="L2" s="71"/>
+      <c r="M2" s="53"/>
+      <c r="N2" s="53"/>
+      <c r="O2" s="55"/>
+      <c r="P2" s="48"/>
+      <c r="Q2" s="61" t="s">
+        <v>2</v>
+      </c>
+      <c r="R2" s="53"/>
+      <c r="S2" s="53"/>
+      <c r="T2" s="77" t="s">
         <v>34</v>
       </c>
-      <c r="AS2" s="61"/>
-      <c r="AT2" s="61"/>
-      <c r="AU2" s="61"/>
-      <c r="AV2" s="60"/>
-      <c r="AW2" s="60"/>
-      <c r="AX2" s="60"/>
-      <c r="AY2" s="60"/>
-      <c r="AZ2" s="58"/>
-      <c r="BA2" s="60" t="s">
-        <v>25</v>
-      </c>
-      <c r="BB2" s="60"/>
-      <c r="BC2" s="60"/>
-      <c r="BD2" s="61" t="s">
+      <c r="U2" s="53"/>
+      <c r="V2" s="53"/>
+      <c r="W2" s="53"/>
+      <c r="X2" s="61"/>
+      <c r="Y2" s="53"/>
+      <c r="Z2" s="53"/>
+      <c r="AA2" s="53"/>
+      <c r="AB2" s="49"/>
+      <c r="AC2" s="61" t="s">
+        <v>2</v>
+      </c>
+      <c r="AD2" s="53"/>
+      <c r="AE2" s="53"/>
+      <c r="AF2" s="77" t="s">
         <v>35</v>
       </c>
-      <c r="BE2" s="61"/>
-      <c r="BF2" s="61"/>
-      <c r="BG2" s="61"/>
-      <c r="BH2" s="60"/>
-      <c r="BI2" s="60"/>
-      <c r="BJ2" s="60"/>
-      <c r="BK2" s="60"/>
-      <c r="BL2" s="53"/>
+      <c r="AG2" s="53"/>
+      <c r="AH2" s="53"/>
+      <c r="AI2" s="53"/>
+      <c r="AJ2" s="61"/>
+      <c r="AK2" s="53"/>
+      <c r="AL2" s="53"/>
+      <c r="AM2" s="53"/>
+      <c r="AN2" s="49"/>
+      <c r="AO2" s="61" t="s">
+        <v>2</v>
+      </c>
+      <c r="AP2" s="53"/>
+      <c r="AQ2" s="53"/>
+      <c r="AR2" s="77" t="s">
+        <v>36</v>
+      </c>
+      <c r="AS2" s="53"/>
+      <c r="AT2" s="53"/>
+      <c r="AU2" s="53"/>
+      <c r="AV2" s="61"/>
+      <c r="AW2" s="53"/>
+      <c r="AX2" s="53"/>
+      <c r="AY2" s="53"/>
+      <c r="AZ2" s="49"/>
+      <c r="BA2" s="61" t="s">
+        <v>2</v>
+      </c>
+      <c r="BB2" s="53"/>
+      <c r="BC2" s="53"/>
+      <c r="BD2" s="77" t="s">
+        <v>37</v>
+      </c>
+      <c r="BE2" s="53"/>
+      <c r="BF2" s="53"/>
+      <c r="BG2" s="53"/>
+      <c r="BH2" s="61"/>
+      <c r="BI2" s="53"/>
+      <c r="BJ2" s="53"/>
+      <c r="BK2" s="93"/>
+      <c r="BL2" s="44"/>
     </row>
     <row r="3" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="79"/>
-      <c r="D3" s="81" t="s">
-        <v>22</v>
-      </c>
-      <c r="E3" s="76"/>
-      <c r="F3" s="72"/>
-      <c r="G3" s="73"/>
-      <c r="H3" s="70"/>
-      <c r="I3" s="71"/>
-      <c r="J3" s="75" t="s">
-        <v>17</v>
-      </c>
-      <c r="K3" s="76"/>
-      <c r="L3" s="72"/>
-      <c r="M3" s="73"/>
-      <c r="N3" s="70"/>
-      <c r="O3" s="71"/>
-      <c r="P3" s="75" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q3" s="76"/>
-      <c r="R3" s="72"/>
-      <c r="S3" s="73"/>
-      <c r="T3" s="70"/>
-      <c r="U3" s="71"/>
-      <c r="V3" s="75" t="s">
-        <v>17</v>
-      </c>
-      <c r="W3" s="76"/>
-      <c r="X3" s="72"/>
-      <c r="Y3" s="73"/>
-      <c r="Z3" s="70"/>
-      <c r="AA3" s="71"/>
-      <c r="AB3" s="77" t="s">
-        <v>22</v>
-      </c>
-      <c r="AC3" s="76"/>
-      <c r="AD3" s="72"/>
-      <c r="AE3" s="73"/>
-      <c r="AF3" s="70"/>
-      <c r="AG3" s="71"/>
-      <c r="AH3" s="75" t="s">
-        <v>17</v>
-      </c>
-      <c r="AI3" s="76"/>
-      <c r="AJ3" s="72"/>
-      <c r="AK3" s="73"/>
-      <c r="AL3" s="70"/>
-      <c r="AM3" s="71"/>
-      <c r="AN3" s="75" t="s">
-        <v>22</v>
-      </c>
-      <c r="AO3" s="76"/>
-      <c r="AP3" s="72"/>
-      <c r="AQ3" s="73"/>
-      <c r="AR3" s="70"/>
-      <c r="AS3" s="71"/>
-      <c r="AT3" s="75" t="s">
-        <v>17</v>
-      </c>
-      <c r="AU3" s="76"/>
-      <c r="AV3" s="72"/>
-      <c r="AW3" s="73"/>
-      <c r="AX3" s="70"/>
-      <c r="AY3" s="71"/>
-      <c r="AZ3" s="75" t="s">
-        <v>22</v>
-      </c>
-      <c r="BA3" s="76"/>
-      <c r="BB3" s="72"/>
-      <c r="BC3" s="73"/>
-      <c r="BD3" s="70"/>
-      <c r="BE3" s="71"/>
-      <c r="BF3" s="75" t="s">
-        <v>17</v>
-      </c>
-      <c r="BG3" s="76"/>
-      <c r="BH3" s="72"/>
-      <c r="BI3" s="73"/>
-      <c r="BJ3" s="70"/>
-      <c r="BK3" s="70"/>
-      <c r="BL3" s="53"/>
-    </row>
-    <row r="4" spans="1:64" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C4" s="80"/>
+        <v>8</v>
+      </c>
+      <c r="C3" s="84"/>
+      <c r="D3" s="82" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="55"/>
+      <c r="F3" s="52"/>
+      <c r="G3" s="53"/>
+      <c r="H3" s="60"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="54" t="s">
+        <v>10</v>
+      </c>
+      <c r="K3" s="55"/>
+      <c r="L3" s="52"/>
+      <c r="M3" s="53"/>
+      <c r="N3" s="60"/>
+      <c r="O3" s="55"/>
+      <c r="P3" s="54" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q3" s="55"/>
+      <c r="R3" s="52"/>
+      <c r="S3" s="53"/>
+      <c r="T3" s="60"/>
+      <c r="U3" s="55"/>
+      <c r="V3" s="54" t="s">
+        <v>10</v>
+      </c>
+      <c r="W3" s="55"/>
+      <c r="X3" s="52"/>
+      <c r="Y3" s="53"/>
+      <c r="Z3" s="60"/>
+      <c r="AA3" s="55"/>
+      <c r="AB3" s="92" t="s">
+        <v>9</v>
+      </c>
+      <c r="AC3" s="55"/>
+      <c r="AD3" s="52"/>
+      <c r="AE3" s="53"/>
+      <c r="AF3" s="60"/>
+      <c r="AG3" s="55"/>
+      <c r="AH3" s="54" t="s">
+        <v>10</v>
+      </c>
+      <c r="AI3" s="55"/>
+      <c r="AJ3" s="52"/>
+      <c r="AK3" s="53"/>
+      <c r="AL3" s="60"/>
+      <c r="AM3" s="55"/>
+      <c r="AN3" s="54" t="s">
+        <v>9</v>
+      </c>
+      <c r="AO3" s="55"/>
+      <c r="AP3" s="52"/>
+      <c r="AQ3" s="53"/>
+      <c r="AR3" s="60"/>
+      <c r="AS3" s="55"/>
+      <c r="AT3" s="54" t="s">
+        <v>10</v>
+      </c>
+      <c r="AU3" s="55"/>
+      <c r="AV3" s="52"/>
+      <c r="AW3" s="53"/>
+      <c r="AX3" s="60"/>
+      <c r="AY3" s="55"/>
+      <c r="AZ3" s="54" t="s">
+        <v>9</v>
+      </c>
+      <c r="BA3" s="55"/>
+      <c r="BB3" s="52"/>
+      <c r="BC3" s="53"/>
+      <c r="BD3" s="60"/>
+      <c r="BE3" s="55"/>
+      <c r="BF3" s="54" t="s">
+        <v>10</v>
+      </c>
+      <c r="BG3" s="55"/>
+      <c r="BH3" s="52"/>
+      <c r="BI3" s="53"/>
+      <c r="BJ3" s="76"/>
+      <c r="BK3" s="93"/>
+      <c r="BL3" s="44"/>
+    </row>
+    <row r="4" spans="1:64" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="51"/>
+      <c r="C4" s="85"/>
       <c r="D4" s="88" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" s="89"/>
-      <c r="F4" s="90"/>
-      <c r="G4" s="91"/>
-      <c r="H4" s="92"/>
-      <c r="I4" s="92"/>
-      <c r="J4" s="92"/>
-      <c r="K4" s="92"/>
-      <c r="L4" s="92"/>
-      <c r="M4" s="92"/>
-      <c r="N4" s="92"/>
-      <c r="O4" s="92"/>
-      <c r="P4" s="93" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q4" s="89"/>
-      <c r="R4" s="90"/>
-      <c r="S4" s="91"/>
-      <c r="T4" s="92"/>
-      <c r="U4" s="92"/>
-      <c r="V4" s="92"/>
-      <c r="W4" s="92"/>
-      <c r="X4" s="92"/>
-      <c r="Y4" s="92"/>
-      <c r="Z4" s="92"/>
-      <c r="AA4" s="94"/>
-      <c r="AB4" s="93" t="s">
-        <v>23</v>
-      </c>
-      <c r="AC4" s="89"/>
-      <c r="AD4" s="90"/>
-      <c r="AE4" s="91"/>
-      <c r="AF4" s="92"/>
-      <c r="AG4" s="92"/>
-      <c r="AH4" s="92"/>
-      <c r="AI4" s="92"/>
-      <c r="AJ4" s="92"/>
-      <c r="AK4" s="92"/>
-      <c r="AL4" s="92"/>
-      <c r="AM4" s="92"/>
-      <c r="AN4" s="93" t="s">
-        <v>23</v>
-      </c>
-      <c r="AO4" s="89"/>
-      <c r="AP4" s="90"/>
-      <c r="AQ4" s="91"/>
-      <c r="AR4" s="92"/>
-      <c r="AS4" s="92"/>
-      <c r="AT4" s="92"/>
-      <c r="AU4" s="92"/>
-      <c r="AV4" s="92"/>
-      <c r="AW4" s="92"/>
-      <c r="AX4" s="92"/>
-      <c r="AY4" s="92"/>
-      <c r="AZ4" s="93" t="s">
-        <v>23</v>
-      </c>
-      <c r="BA4" s="89"/>
-      <c r="BB4" s="90"/>
-      <c r="BC4" s="91"/>
-      <c r="BD4" s="92"/>
-      <c r="BE4" s="92"/>
-      <c r="BF4" s="92"/>
-      <c r="BG4" s="92"/>
-      <c r="BH4" s="92"/>
-      <c r="BI4" s="92"/>
-      <c r="BJ4" s="92"/>
-      <c r="BK4" s="96"/>
+        <v>11</v>
+      </c>
+      <c r="E4" s="66"/>
+      <c r="F4" s="67"/>
+      <c r="G4" s="79"/>
+      <c r="H4" s="66"/>
+      <c r="I4" s="66"/>
+      <c r="J4" s="66"/>
+      <c r="K4" s="66"/>
+      <c r="L4" s="66"/>
+      <c r="M4" s="66"/>
+      <c r="N4" s="66"/>
+      <c r="O4" s="66"/>
+      <c r="P4" s="68" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q4" s="66"/>
+      <c r="R4" s="67"/>
+      <c r="S4" s="65"/>
+      <c r="T4" s="66"/>
+      <c r="U4" s="66"/>
+      <c r="V4" s="66"/>
+      <c r="W4" s="66"/>
+      <c r="X4" s="66"/>
+      <c r="Y4" s="66"/>
+      <c r="Z4" s="66"/>
+      <c r="AA4" s="67"/>
+      <c r="AB4" s="68" t="s">
+        <v>11</v>
+      </c>
+      <c r="AC4" s="66"/>
+      <c r="AD4" s="67"/>
+      <c r="AE4" s="79"/>
+      <c r="AF4" s="66"/>
+      <c r="AG4" s="66"/>
+      <c r="AH4" s="66"/>
+      <c r="AI4" s="66"/>
+      <c r="AJ4" s="66"/>
+      <c r="AK4" s="66"/>
+      <c r="AL4" s="66"/>
+      <c r="AM4" s="66"/>
+      <c r="AN4" s="68" t="s">
+        <v>11</v>
+      </c>
+      <c r="AO4" s="66"/>
+      <c r="AP4" s="67"/>
+      <c r="AQ4" s="79"/>
+      <c r="AR4" s="66"/>
+      <c r="AS4" s="66"/>
+      <c r="AT4" s="66"/>
+      <c r="AU4" s="66"/>
+      <c r="AV4" s="66"/>
+      <c r="AW4" s="66"/>
+      <c r="AX4" s="66"/>
+      <c r="AY4" s="66"/>
+      <c r="AZ4" s="68" t="s">
+        <v>11</v>
+      </c>
+      <c r="BA4" s="66"/>
+      <c r="BB4" s="67"/>
+      <c r="BC4" s="80"/>
+      <c r="BD4" s="66"/>
+      <c r="BE4" s="66"/>
+      <c r="BF4" s="66"/>
+      <c r="BG4" s="66"/>
+      <c r="BH4" s="66"/>
+      <c r="BI4" s="66"/>
+      <c r="BJ4" s="66"/>
+      <c r="BK4" s="81"/>
     </row>
     <row r="5" spans="1:64" ht="20.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="59"/>
+      <c r="B5" s="25"/>
       <c r="C5" s="2"/>
       <c r="D5" s="11">
         <v>1</v>
@@ -3965,25 +3971,25 @@
         <v>4</v>
       </c>
       <c r="H5" s="12" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="I5" s="12">
         <v>5</v>
       </c>
       <c r="J5" s="12" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="K5" s="12">
         <v>6</v>
       </c>
       <c r="L5" s="12" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="M5" s="12">
         <v>7</v>
       </c>
       <c r="N5" s="12" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="O5" s="13">
         <v>8</v>
@@ -4001,25 +4007,25 @@
         <v>4</v>
       </c>
       <c r="T5" s="12" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="U5" s="12">
         <v>5</v>
       </c>
       <c r="V5" s="12" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="W5" s="12">
         <v>6</v>
       </c>
       <c r="X5" s="12" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="Y5" s="12">
         <v>7</v>
       </c>
       <c r="Z5" s="12" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="AA5" s="13">
         <v>8</v>
@@ -4037,25 +4043,25 @@
         <v>4</v>
       </c>
       <c r="AF5" s="12" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="AG5" s="12">
         <v>5</v>
       </c>
       <c r="AH5" s="12" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="AI5" s="12">
         <v>6</v>
       </c>
       <c r="AJ5" s="12" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="AK5" s="12">
         <v>7</v>
       </c>
       <c r="AL5" s="12" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="AM5" s="13">
         <v>8</v>
@@ -4073,25 +4079,25 @@
         <v>4</v>
       </c>
       <c r="AR5" s="12" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="AS5" s="12">
         <v>5</v>
       </c>
       <c r="AT5" s="12" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="AU5" s="12">
         <v>6</v>
       </c>
       <c r="AV5" s="12" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="AW5" s="12">
         <v>7</v>
       </c>
       <c r="AX5" s="12" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="AY5" s="13">
         <v>8</v>
@@ -4109,25 +4115,25 @@
         <v>4</v>
       </c>
       <c r="BD5" s="12" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="BE5" s="12">
         <v>5</v>
       </c>
       <c r="BF5" s="12" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="BG5" s="12">
         <v>6</v>
       </c>
       <c r="BH5" s="12" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="BI5" s="12">
         <v>7</v>
       </c>
       <c r="BJ5" s="12" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="BK5" s="14">
         <v>8</v>
@@ -4138,7 +4144,7 @@
         <v>1</v>
       </c>
       <c r="C6" s="28" t="s">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="D6" s="31"/>
       <c r="E6" s="18"/>
@@ -5328,118 +5334,118 @@
         <v>19</v>
       </c>
       <c r="C24" s="27"/>
-      <c r="D24" s="44"/>
-      <c r="E24" s="45"/>
-      <c r="F24" s="46"/>
-      <c r="G24" s="47"/>
-      <c r="H24" s="48"/>
-      <c r="I24" s="49"/>
-      <c r="J24" s="45"/>
-      <c r="K24" s="50"/>
-      <c r="L24" s="46"/>
-      <c r="M24" s="46"/>
-      <c r="N24" s="51"/>
-      <c r="O24" s="51"/>
-      <c r="P24" s="44"/>
-      <c r="Q24" s="45"/>
-      <c r="R24" s="46"/>
-      <c r="S24" s="47"/>
-      <c r="T24" s="48"/>
-      <c r="U24" s="49"/>
-      <c r="V24" s="45"/>
-      <c r="W24" s="50"/>
-      <c r="X24" s="46"/>
-      <c r="Y24" s="46"/>
-      <c r="Z24" s="51"/>
-      <c r="AA24" s="51"/>
-      <c r="AB24" s="44"/>
-      <c r="AC24" s="45"/>
-      <c r="AD24" s="46"/>
-      <c r="AE24" s="47"/>
-      <c r="AF24" s="48"/>
-      <c r="AG24" s="49"/>
-      <c r="AH24" s="45"/>
-      <c r="AI24" s="50"/>
-      <c r="AJ24" s="46"/>
-      <c r="AK24" s="46"/>
-      <c r="AL24" s="51"/>
-      <c r="AM24" s="51"/>
-      <c r="AN24" s="44"/>
-      <c r="AO24" s="45"/>
-      <c r="AP24" s="46"/>
-      <c r="AQ24" s="47"/>
-      <c r="AR24" s="48"/>
-      <c r="AS24" s="49"/>
-      <c r="AT24" s="45"/>
-      <c r="AU24" s="50"/>
-      <c r="AV24" s="46"/>
-      <c r="AW24" s="46"/>
-      <c r="AX24" s="51"/>
-      <c r="AY24" s="51"/>
-      <c r="AZ24" s="44"/>
-      <c r="BA24" s="45"/>
-      <c r="BB24" s="46"/>
-      <c r="BC24" s="47"/>
-      <c r="BD24" s="48"/>
-      <c r="BE24" s="49"/>
-      <c r="BF24" s="45"/>
-      <c r="BG24" s="50"/>
-      <c r="BH24" s="46"/>
-      <c r="BI24" s="46"/>
-      <c r="BJ24" s="51"/>
-      <c r="BK24" s="52"/>
-    </row>
-    <row r="25" spans="2:63" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D24" s="31"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="32"/>
+      <c r="G24" s="33"/>
+      <c r="H24" s="34"/>
+      <c r="I24" s="35"/>
+      <c r="J24" s="18"/>
+      <c r="K24" s="19"/>
+      <c r="L24" s="32"/>
+      <c r="M24" s="32"/>
+      <c r="N24" s="36"/>
+      <c r="O24" s="36"/>
+      <c r="P24" s="31"/>
+      <c r="Q24" s="18"/>
+      <c r="R24" s="32"/>
+      <c r="S24" s="33"/>
+      <c r="T24" s="34"/>
+      <c r="U24" s="35"/>
+      <c r="V24" s="18"/>
+      <c r="W24" s="19"/>
+      <c r="X24" s="32"/>
+      <c r="Y24" s="32"/>
+      <c r="Z24" s="36"/>
+      <c r="AA24" s="36"/>
+      <c r="AB24" s="31"/>
+      <c r="AC24" s="18"/>
+      <c r="AD24" s="32"/>
+      <c r="AE24" s="33"/>
+      <c r="AF24" s="34"/>
+      <c r="AG24" s="35"/>
+      <c r="AH24" s="18"/>
+      <c r="AI24" s="19"/>
+      <c r="AJ24" s="32"/>
+      <c r="AK24" s="32"/>
+      <c r="AL24" s="36"/>
+      <c r="AM24" s="36"/>
+      <c r="AN24" s="31"/>
+      <c r="AO24" s="18"/>
+      <c r="AP24" s="32"/>
+      <c r="AQ24" s="33"/>
+      <c r="AR24" s="34"/>
+      <c r="AS24" s="35"/>
+      <c r="AT24" s="18"/>
+      <c r="AU24" s="19"/>
+      <c r="AV24" s="32"/>
+      <c r="AW24" s="32"/>
+      <c r="AX24" s="36"/>
+      <c r="AY24" s="36"/>
+      <c r="AZ24" s="31"/>
+      <c r="BA24" s="18"/>
+      <c r="BB24" s="32"/>
+      <c r="BC24" s="33"/>
+      <c r="BD24" s="34"/>
+      <c r="BE24" s="35"/>
+      <c r="BF24" s="18"/>
+      <c r="BG24" s="19"/>
+      <c r="BH24" s="32"/>
+      <c r="BI24" s="32"/>
+      <c r="BJ24" s="36"/>
+      <c r="BK24" s="37"/>
+    </row>
+    <row r="25" spans="2:63" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C25" s="42" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D25" s="7"/>
       <c r="O25" s="8"/>
-      <c r="P25" s="85" t="s">
+      <c r="P25" s="56" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q25" s="57"/>
+      <c r="R25" s="57"/>
+      <c r="S25" s="57"/>
+      <c r="T25" s="57"/>
+      <c r="U25" s="57"/>
+      <c r="V25" s="57"/>
+      <c r="W25" s="57"/>
+      <c r="X25" s="57"/>
+      <c r="Y25" s="57"/>
+      <c r="Z25" s="57"/>
+      <c r="AA25" s="58"/>
+      <c r="AB25" s="56" t="s">
         <v>19</v>
       </c>
-      <c r="Q25" s="86"/>
-      <c r="R25" s="86"/>
-      <c r="S25" s="86"/>
-      <c r="T25" s="86"/>
-      <c r="U25" s="86"/>
-      <c r="V25" s="86"/>
-      <c r="W25" s="86"/>
-      <c r="X25" s="86"/>
-      <c r="Y25" s="86"/>
-      <c r="Z25" s="86"/>
-      <c r="AA25" s="87"/>
-      <c r="AB25" s="85" t="s">
-        <v>18</v>
-      </c>
-      <c r="AC25" s="86"/>
-      <c r="AD25" s="86"/>
-      <c r="AE25" s="86"/>
-      <c r="AF25" s="86"/>
-      <c r="AG25" s="86"/>
-      <c r="AH25" s="86"/>
-      <c r="AI25" s="86"/>
-      <c r="AJ25" s="86"/>
-      <c r="AK25" s="86"/>
-      <c r="AL25" s="86"/>
-      <c r="AM25" s="87"/>
+      <c r="AC25" s="57"/>
+      <c r="AD25" s="57"/>
+      <c r="AE25" s="57"/>
+      <c r="AF25" s="57"/>
+      <c r="AG25" s="57"/>
+      <c r="AH25" s="57"/>
+      <c r="AI25" s="57"/>
+      <c r="AJ25" s="57"/>
+      <c r="AK25" s="57"/>
+      <c r="AL25" s="57"/>
+      <c r="AM25" s="58"/>
       <c r="AZ25" s="7"/>
       <c r="BK25" s="5"/>
     </row>
     <row r="26" spans="2:63" x14ac:dyDescent="0.25">
-      <c r="C26" s="54" t="s">
-        <v>24</v>
-      </c>
-      <c r="D26" s="68"/>
-      <c r="E26" s="69"/>
+      <c r="C26" s="45" t="s">
+        <v>21</v>
+      </c>
+      <c r="D26" s="69"/>
+      <c r="E26" s="55"/>
       <c r="O26" s="8"/>
-      <c r="P26" s="68"/>
-      <c r="Q26" s="69"/>
-      <c r="AB26" s="68"/>
-      <c r="AC26" s="69"/>
+      <c r="P26" s="69"/>
+      <c r="Q26" s="55"/>
+      <c r="AB26" s="69"/>
+      <c r="AC26" s="55"/>
       <c r="AM26" s="8"/>
-      <c r="AN26" s="68"/>
-      <c r="AO26" s="69"/>
+      <c r="AN26" s="69"/>
+      <c r="AO26" s="55"/>
       <c r="AP26" s="21"/>
       <c r="AQ26" s="21"/>
       <c r="AR26" s="21"/>
@@ -5450,46 +5456,46 @@
       <c r="AW26" s="21"/>
       <c r="AX26" s="21"/>
       <c r="AY26" s="30"/>
-      <c r="AZ26" s="68"/>
-      <c r="BA26" s="69"/>
+      <c r="AZ26" s="69"/>
+      <c r="BA26" s="55"/>
       <c r="BK26" s="5"/>
     </row>
     <row r="27" spans="2:63" x14ac:dyDescent="0.25">
       <c r="C27" s="40" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="D27" s="20"/>
       <c r="E27" s="3"/>
       <c r="O27" s="8"/>
       <c r="P27" s="17"/>
       <c r="Q27" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="S27" s="95" t="s">
-        <v>20</v>
-      </c>
-      <c r="T27" s="95"/>
-      <c r="U27" s="95"/>
-      <c r="V27" s="95"/>
-      <c r="W27" s="95"/>
-      <c r="X27" s="95"/>
-      <c r="Y27" s="95"/>
-      <c r="Z27" s="95"/>
+        <v>25</v>
+      </c>
+      <c r="S27" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="T27" s="57"/>
+      <c r="U27" s="57"/>
+      <c r="V27" s="57"/>
+      <c r="W27" s="57"/>
+      <c r="X27" s="57"/>
+      <c r="Y27" s="57"/>
+      <c r="Z27" s="57"/>
       <c r="AA27" s="8"/>
       <c r="AB27" s="17"/>
       <c r="AC27" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="AE27" s="95" t="s">
-        <v>20</v>
-      </c>
-      <c r="AF27" s="95"/>
-      <c r="AG27" s="95"/>
-      <c r="AH27" s="95"/>
-      <c r="AI27" s="95"/>
-      <c r="AJ27" s="95"/>
-      <c r="AK27" s="95"/>
-      <c r="AL27" s="95"/>
+        <v>23</v>
+      </c>
+      <c r="AE27" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="AF27" s="57"/>
+      <c r="AG27" s="57"/>
+      <c r="AH27" s="57"/>
+      <c r="AI27" s="57"/>
+      <c r="AJ27" s="57"/>
+      <c r="AK27" s="57"/>
+      <c r="AL27" s="57"/>
       <c r="AM27" s="8"/>
       <c r="AN27" s="20"/>
       <c r="AO27" s="3"/>
@@ -5499,7 +5505,7 @@
     </row>
     <row r="28" spans="2:63" x14ac:dyDescent="0.25">
       <c r="C28" s="40" t="s">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="D28" s="15"/>
       <c r="E28" s="3"/>
@@ -5518,14 +5524,14 @@
     </row>
     <row r="29" spans="2:63" x14ac:dyDescent="0.25">
       <c r="C29" s="40" t="s">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="D29" s="1"/>
       <c r="E29" s="3"/>
       <c r="O29" s="8"/>
       <c r="P29" s="1"/>
       <c r="Q29" s="22" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="R29" s="21"/>
       <c r="S29" s="21"/>
@@ -5533,7 +5539,7 @@
       <c r="AA29" s="8"/>
       <c r="AB29" s="1"/>
       <c r="AC29" s="22" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="AD29" s="21"/>
       <c r="AE29" s="21"/>
@@ -5547,7 +5553,7 @@
     </row>
     <row r="30" spans="2:63" x14ac:dyDescent="0.25">
       <c r="C30" s="40" t="s">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="D30" s="1"/>
       <c r="E30" s="3"/>
@@ -5564,9 +5570,9 @@
       <c r="BA30" s="3"/>
       <c r="BK30" s="5"/>
     </row>
-    <row r="31" spans="2:63" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:63" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C31" s="41" t="s">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="D31" s="16"/>
       <c r="E31" s="10"/>
@@ -5629,96 +5635,87 @@
       <c r="BJ31" s="4"/>
       <c r="BK31" s="6"/>
     </row>
-    <row r="32" spans="2:63" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="2:63" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="75">
+    <mergeCell ref="AE27:AL27"/>
+    <mergeCell ref="T3:U3"/>
+    <mergeCell ref="AF2:AI2"/>
+    <mergeCell ref="V3:W3"/>
+    <mergeCell ref="AB3:AC3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="BD2:BG2"/>
+    <mergeCell ref="AN1:AT1"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="BH2:BK2"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="AX3:AY3"/>
+    <mergeCell ref="P3:Q3"/>
+    <mergeCell ref="BJ3:BK3"/>
+    <mergeCell ref="AZ3:BA3"/>
+    <mergeCell ref="AO2:AQ2"/>
+    <mergeCell ref="BA2:BC2"/>
+    <mergeCell ref="H2:K2"/>
+    <mergeCell ref="T2:W2"/>
+    <mergeCell ref="AR3:AS3"/>
+    <mergeCell ref="BH3:BI3"/>
+    <mergeCell ref="AN26:AO26"/>
+    <mergeCell ref="N3:O3"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="K1:O1"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="AN4:AP4"/>
+    <mergeCell ref="L2:O2"/>
+    <mergeCell ref="W1:AA1"/>
+    <mergeCell ref="X2:AA2"/>
+    <mergeCell ref="BG1:BK1"/>
+    <mergeCell ref="AQ4:AY4"/>
+    <mergeCell ref="D1:J1"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="P1:V1"/>
+    <mergeCell ref="G4:O4"/>
+    <mergeCell ref="BD3:BE3"/>
+    <mergeCell ref="AT3:AU3"/>
+    <mergeCell ref="BF3:BG3"/>
+    <mergeCell ref="AV3:AW3"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="X3:Y3"/>
+    <mergeCell ref="Z3:AA3"/>
+    <mergeCell ref="AJ3:AK3"/>
+    <mergeCell ref="AL3:AM3"/>
+    <mergeCell ref="R3:S3"/>
     <mergeCell ref="C1:C4"/>
     <mergeCell ref="S27:Z27"/>
-    <mergeCell ref="AE27:AL27"/>
+    <mergeCell ref="AZ4:BB4"/>
+    <mergeCell ref="AU1:AY1"/>
+    <mergeCell ref="AB26:AC26"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="AZ1:BF1"/>
+    <mergeCell ref="Q2:S2"/>
+    <mergeCell ref="BC4:BK4"/>
+    <mergeCell ref="AJ2:AM2"/>
+    <mergeCell ref="AZ26:BA26"/>
+    <mergeCell ref="AC2:AE2"/>
+    <mergeCell ref="AB1:AH1"/>
+    <mergeCell ref="S4:AA4"/>
     <mergeCell ref="AE4:AM4"/>
-    <mergeCell ref="AN4:AP4"/>
-    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="AV2:AY2"/>
+    <mergeCell ref="AN3:AO3"/>
+    <mergeCell ref="AP3:AQ3"/>
+    <mergeCell ref="BB3:BC3"/>
+    <mergeCell ref="AI1:AM1"/>
+    <mergeCell ref="AR2:AU2"/>
+    <mergeCell ref="AD3:AE3"/>
     <mergeCell ref="P26:Q26"/>
-    <mergeCell ref="AB26:AC26"/>
-    <mergeCell ref="AN26:AO26"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="G4:O4"/>
+    <mergeCell ref="AF3:AG3"/>
+    <mergeCell ref="AH3:AI3"/>
+    <mergeCell ref="AB25:AM25"/>
     <mergeCell ref="P4:R4"/>
-    <mergeCell ref="S4:AA4"/>
+    <mergeCell ref="P25:AA25"/>
     <mergeCell ref="AB4:AD4"/>
-    <mergeCell ref="BH3:BI3"/>
-    <mergeCell ref="BJ3:BK3"/>
-    <mergeCell ref="AZ4:BB4"/>
-    <mergeCell ref="BC4:BK4"/>
-    <mergeCell ref="P25:AA25"/>
-    <mergeCell ref="AB25:AM25"/>
-    <mergeCell ref="AQ4:AY4"/>
-    <mergeCell ref="AZ3:BA3"/>
-    <mergeCell ref="BF3:BG3"/>
-    <mergeCell ref="AV3:AW3"/>
-    <mergeCell ref="AX3:AY3"/>
-    <mergeCell ref="BB3:BC3"/>
-    <mergeCell ref="BD3:BE3"/>
-    <mergeCell ref="AT3:AU3"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="P3:Q3"/>
-    <mergeCell ref="V3:W3"/>
-    <mergeCell ref="AB3:AC3"/>
-    <mergeCell ref="AH3:AI3"/>
-    <mergeCell ref="AN3:AO3"/>
-    <mergeCell ref="AJ3:AK3"/>
-    <mergeCell ref="AL3:AM3"/>
-    <mergeCell ref="AP3:AQ3"/>
-    <mergeCell ref="AR3:AS3"/>
-    <mergeCell ref="BD2:BG2"/>
-    <mergeCell ref="BH2:BK2"/>
-    <mergeCell ref="D1:J1"/>
-    <mergeCell ref="K1:O1"/>
-    <mergeCell ref="P1:V1"/>
-    <mergeCell ref="W1:AA1"/>
-    <mergeCell ref="AB1:AH1"/>
-    <mergeCell ref="AI1:AM1"/>
-    <mergeCell ref="AN1:AT1"/>
-    <mergeCell ref="AU1:AY1"/>
-    <mergeCell ref="AZ1:BF1"/>
-    <mergeCell ref="X3:Y3"/>
-    <mergeCell ref="Z3:AA3"/>
-    <mergeCell ref="AD3:AE3"/>
-    <mergeCell ref="AF3:AG3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="N3:O3"/>
-    <mergeCell ref="R3:S3"/>
-    <mergeCell ref="BG1:BK1"/>
-    <mergeCell ref="AZ26:BA26"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="H2:K2"/>
-    <mergeCell ref="L2:O2"/>
-    <mergeCell ref="Q2:S2"/>
-    <mergeCell ref="T2:W2"/>
-    <mergeCell ref="X2:AA2"/>
-    <mergeCell ref="AC2:AE2"/>
-    <mergeCell ref="AF2:AI2"/>
-    <mergeCell ref="AJ2:AM2"/>
-    <mergeCell ref="AO2:AQ2"/>
-    <mergeCell ref="AR2:AU2"/>
-    <mergeCell ref="AV2:AY2"/>
-    <mergeCell ref="BA2:BC2"/>
-    <mergeCell ref="T3:U3"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0" footer="0"/>
   <pageSetup orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBFF96AB-D91B-4FA7-AD0E-30F370406C6C}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>